<commit_message>
Add XING DONG 88 MGO=1.2mt/d in Sheet4
</commit_message>
<xml_diff>
--- a/Port Distance.xlsx
+++ b/Port Distance.xlsx
@@ -11694,6 +11694,9 @@
       <c r="E265" s="5" t="n">
         <v>12.5</v>
       </c>
+      <c r="F265" t="n">
+        <v>1.2</v>
+      </c>
     </row>
     <row r="266">
       <c r="A266" s="7" t="inlineStr">
@@ -11712,6 +11715,9 @@
       <c r="E266" s="5" t="n">
         <v>15.5</v>
       </c>
+      <c r="F266" t="n">
+        <v>1.2</v>
+      </c>
     </row>
     <row r="267">
       <c r="A267" s="7" t="inlineStr">
@@ -11729,6 +11735,9 @@
       </c>
       <c r="E267" s="5" t="n">
         <v>18</v>
+      </c>
+      <c r="F267" t="n">
+        <v>1.2</v>
       </c>
     </row>
     <row r="268">
@@ -12008,56 +12017,56 @@
       </c>
     </row>
     <row r="284">
-      <c r="A284" t="inlineStr">
+      <c r="A284" s="0" t="inlineStr">
         <is>
           <t>KR TASMAN</t>
         </is>
       </c>
-      <c r="B284" t="inlineStr">
+      <c r="B284" s="0" t="inlineStr">
         <is>
           <t>KRTM</t>
         </is>
       </c>
-      <c r="C284" t="n">
+      <c r="C284" s="0" t="n">
         <v>15</v>
       </c>
-      <c r="E284" t="n">
+      <c r="E284" s="0" t="n">
         <v>35</v>
       </c>
     </row>
     <row r="285">
-      <c r="A285" t="inlineStr">
+      <c r="A285" s="0" t="inlineStr">
         <is>
           <t>KR TASMAN</t>
         </is>
       </c>
-      <c r="B285" t="inlineStr">
+      <c r="B285" s="0" t="inlineStr">
         <is>
           <t>KRTM</t>
         </is>
       </c>
-      <c r="C285" t="n">
+      <c r="C285" s="0" t="n">
         <v>15.5</v>
       </c>
-      <c r="E285" t="n">
+      <c r="E285" s="0" t="n">
         <v>38</v>
       </c>
     </row>
     <row r="286">
-      <c r="A286" t="inlineStr">
+      <c r="A286" s="0" t="inlineStr">
         <is>
           <t>KR TASMAN</t>
         </is>
       </c>
-      <c r="B286" t="inlineStr">
+      <c r="B286" s="0" t="inlineStr">
         <is>
           <t>KRTM</t>
         </is>
       </c>
-      <c r="C286" t="n">
+      <c r="C286" s="0" t="n">
         <v>16</v>
       </c>
-      <c r="E286" t="n">
+      <c r="E286" s="0" t="n">
         <v>42</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add NOBAL STAR vessel data and CSV distances/ports/vessels files
</commit_message>
<xml_diff>
--- a/Port Distance.xlsx
+++ b/Port Distance.xlsx
@@ -1276,13 +1276,13 @@
       <c r="AF3" s="20" t="n"/>
       <c r="AG3" s="39" t="n"/>
       <c r="AH3" s="40" t="n">
-        <v>3641</v>
+        <v>5809.8</v>
       </c>
       <c r="AI3" s="40" t="n">
-        <v>5430</v>
+        <v>8503.450000000001</v>
       </c>
       <c r="AJ3" s="40" t="n">
-        <v>5736</v>
+        <v>9083.51</v>
       </c>
     </row>
     <row r="4" ht="15.6" customHeight="1" s="37">
@@ -1292,7 +1292,7 @@
         </is>
       </c>
       <c r="B4" s="11" t="n">
-        <v>357</v>
+        <v>386.8</v>
       </c>
       <c r="C4" s="20" t="n"/>
       <c r="D4" s="20" t="n"/>
@@ -1326,13 +1326,13 @@
       <c r="AF4" s="20" t="n"/>
       <c r="AG4" s="39" t="n"/>
       <c r="AH4" s="40" t="n">
-        <v>3754</v>
+        <v>5539.6</v>
       </c>
       <c r="AI4" s="40" t="n">
-        <v>5664</v>
+        <v>8230.93</v>
       </c>
       <c r="AJ4" s="40" t="n">
-        <v>6004</v>
+        <v>8810.98</v>
       </c>
     </row>
     <row r="5" ht="15.6" customHeight="1" s="37">
@@ -1342,10 +1342,10 @@
         </is>
       </c>
       <c r="B5" s="11" t="n">
-        <v>504</v>
+        <v>462.13</v>
       </c>
       <c r="C5" s="23" t="n">
-        <v>200</v>
+        <v>146.77</v>
       </c>
       <c r="D5" s="20" t="n"/>
       <c r="E5" s="20" t="n"/>
@@ -1378,13 +1378,13 @@
       <c r="AF5" s="20" t="n"/>
       <c r="AG5" s="39" t="n"/>
       <c r="AH5" s="40" t="n">
-        <v>3777</v>
+        <v>5386.5</v>
       </c>
       <c r="AI5" s="40" t="n">
-        <v>5720</v>
+        <v>8089.3</v>
       </c>
       <c r="AJ5" s="40" t="n">
-        <v>6071</v>
+        <v>8669.360000000001</v>
       </c>
     </row>
     <row r="6" ht="15.6" customHeight="1" s="37">
@@ -1432,7 +1432,7 @@
       <c r="AF6" s="20" t="n"/>
       <c r="AG6" s="39" t="n"/>
       <c r="AH6" s="40" t="n">
-        <v>3664</v>
+        <v>4879.1</v>
       </c>
       <c r="AI6" s="40" t="n">
         <v>5758</v>
@@ -1448,10 +1448,10 @@
         </is>
       </c>
       <c r="B7" s="11" t="n">
-        <v>1122</v>
+        <v>1153.65</v>
       </c>
       <c r="C7" s="11" t="n">
-        <v>831</v>
+        <v>858.73</v>
       </c>
       <c r="D7" s="11" t="n">
         <v>708</v>
@@ -1488,13 +1488,13 @@
       <c r="AF7" s="20" t="n"/>
       <c r="AG7" s="39" t="n"/>
       <c r="AH7" s="40" t="n">
-        <v>3477</v>
+        <v>4761.6</v>
       </c>
       <c r="AI7" s="40" t="n">
-        <v>5641</v>
+        <v>7481.7</v>
       </c>
       <c r="AJ7" s="40" t="n">
-        <v>6093</v>
+        <v>8061.75</v>
       </c>
     </row>
     <row r="8" ht="15.6" customHeight="1" s="37">
@@ -1504,19 +1504,19 @@
         </is>
       </c>
       <c r="B8" s="11" t="n">
-        <v>1150</v>
+        <v>1171.54</v>
       </c>
       <c r="C8" s="11" t="n">
-        <v>847</v>
+        <v>874.55</v>
       </c>
       <c r="D8" s="11" t="n">
-        <v>736</v>
+        <v>754.38</v>
       </c>
       <c r="E8" s="11" t="n">
         <v>206</v>
       </c>
       <c r="F8" s="23" t="n">
-        <v>60</v>
+        <v>19.16</v>
       </c>
       <c r="G8" s="20" t="n"/>
       <c r="H8" s="20" t="n"/>
@@ -1546,13 +1546,13 @@
       <c r="AF8" s="20" t="n"/>
       <c r="AG8" s="39" t="n"/>
       <c r="AH8" s="40" t="n">
-        <v>3430</v>
+        <v>4771</v>
       </c>
       <c r="AI8" s="40" t="n">
-        <v>5595</v>
+        <v>7485.87</v>
       </c>
       <c r="AJ8" s="40" t="n">
-        <v>6049</v>
+        <v>8065.93</v>
       </c>
     </row>
     <row r="9" ht="15.6" customHeight="1" s="37">
@@ -1606,7 +1606,7 @@
       <c r="AF9" s="20" t="n"/>
       <c r="AG9" s="39" t="n"/>
       <c r="AH9" s="40" t="n">
-        <v>3431</v>
+        <v>4907.3</v>
       </c>
       <c r="AI9" s="40" t="n">
         <v>5594</v>
@@ -1622,19 +1622,19 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>1164</v>
+        <v>1193.2</v>
       </c>
       <c r="C10" s="11" t="n">
-        <v>861</v>
+        <v>896.2</v>
       </c>
       <c r="D10" s="11" t="n">
-        <v>750</v>
+        <v>763.91</v>
       </c>
       <c r="E10" s="11" t="n">
         <v>217</v>
       </c>
       <c r="F10" s="11" t="n">
-        <v>27</v>
+        <v>29.65</v>
       </c>
       <c r="G10" s="11" t="n">
         <v>15</v>
@@ -1668,13 +1668,13 @@
       <c r="AF10" s="20" t="n"/>
       <c r="AG10" s="39" t="n"/>
       <c r="AH10" s="40" t="n">
-        <v>3424</v>
+        <v>4781.6</v>
       </c>
       <c r="AI10" s="40" t="n">
-        <v>5582</v>
+        <v>7497.93</v>
       </c>
       <c r="AJ10" s="40" t="n">
-        <v>6034</v>
+        <v>8077.99</v>
       </c>
     </row>
     <row r="11" ht="15.6" customHeight="1" s="37">
@@ -1732,7 +1732,7 @@
       <c r="AF11" s="20" t="n"/>
       <c r="AG11" s="39" t="n"/>
       <c r="AH11" s="40" t="n">
-        <v>3472</v>
+        <v>4766.3</v>
       </c>
       <c r="AI11" s="40" t="n">
         <v>5641</v>
@@ -1798,7 +1798,7 @@
       <c r="AF12" s="20" t="n"/>
       <c r="AG12" s="39" t="n"/>
       <c r="AH12" s="40" t="n">
-        <v>3856</v>
+        <v>5128.4</v>
       </c>
       <c r="AI12" s="40" t="n">
         <v>5907</v>
@@ -1866,7 +1866,7 @@
       <c r="AF13" s="20" t="n"/>
       <c r="AG13" s="39" t="n"/>
       <c r="AH13" s="40" t="n">
-        <v>3864</v>
+        <v>5128.4</v>
       </c>
       <c r="AI13" s="40" t="n">
         <v>5912</v>
@@ -1936,7 +1936,7 @@
       <c r="AF14" s="20" t="n"/>
       <c r="AG14" s="39" t="n"/>
       <c r="AH14" s="40" t="n">
-        <v>3811</v>
+        <v>5036</v>
       </c>
       <c r="AI14" s="40" t="n">
         <v>5888</v>
@@ -2008,7 +2008,7 @@
       <c r="AF15" s="20" t="n"/>
       <c r="AG15" s="39" t="n"/>
       <c r="AH15" s="40" t="n">
-        <v>3828</v>
+        <v>4936.2</v>
       </c>
       <c r="AI15" s="40" t="n">
         <v>5939</v>
@@ -2082,7 +2082,7 @@
       <c r="AF16" s="20" t="n"/>
       <c r="AG16" s="39" t="n"/>
       <c r="AH16" s="40" t="n">
-        <v>3284</v>
+        <v>3976</v>
       </c>
       <c r="AI16" s="40" t="n">
         <v>5652</v>
@@ -2101,7 +2101,7 @@
         <v>2497</v>
       </c>
       <c r="C17" s="11" t="n">
-        <v>2191</v>
+        <v>2218.83</v>
       </c>
       <c r="D17" s="11" t="n">
         <v>2081</v>
@@ -2158,13 +2158,13 @@
       <c r="AF17" s="20" t="n"/>
       <c r="AG17" s="39" t="n"/>
       <c r="AH17" s="40" t="n">
-        <v>2879</v>
+        <v>4141.6</v>
       </c>
       <c r="AI17" s="40" t="n">
-        <v>5253</v>
+        <v>6757.42</v>
       </c>
       <c r="AJ17" s="40" t="n">
-        <v>5834</v>
+        <v>7385.73</v>
       </c>
     </row>
     <row r="18" ht="15.6" customHeight="1" s="37">
@@ -2236,7 +2236,7 @@
       <c r="AF18" s="20" t="n"/>
       <c r="AG18" s="39" t="n"/>
       <c r="AH18" s="40" t="n">
-        <v>2840</v>
+        <v>4214.8</v>
       </c>
       <c r="AI18" s="40" t="n">
         <v>5210</v>
@@ -2316,7 +2316,7 @@
       <c r="AF19" s="20" t="n"/>
       <c r="AG19" s="39" t="n"/>
       <c r="AH19" s="40" t="n">
-        <v>2847</v>
+        <v>4198</v>
       </c>
       <c r="AI19" s="40" t="n">
         <v>5219</v>
@@ -2398,7 +2398,7 @@
       <c r="AF20" s="20" t="n"/>
       <c r="AG20" s="39" t="n"/>
       <c r="AH20" s="40" t="n">
-        <v>2848</v>
+        <v>3838</v>
       </c>
       <c r="AI20" s="40" t="n">
         <v>5220</v>
@@ -2417,7 +2417,7 @@
         <v>2461</v>
       </c>
       <c r="C21" s="11" t="n">
-        <v>2161</v>
+        <v>2188.37</v>
       </c>
       <c r="D21" s="11" t="n">
         <v>2047</v>
@@ -2456,7 +2456,7 @@
         <v>639</v>
       </c>
       <c r="P21" s="11" t="n">
-        <v>861</v>
+        <v>822.65</v>
       </c>
       <c r="Q21" s="11" t="n">
         <v>854</v>
@@ -2482,13 +2482,13 @@
       <c r="AF21" s="21" t="n"/>
       <c r="AG21" s="39" t="n"/>
       <c r="AH21" s="40" t="n">
-        <v>3415</v>
+        <v>3310.7</v>
       </c>
       <c r="AI21" s="40" t="n">
-        <v>5830</v>
+        <v>5926.6</v>
       </c>
       <c r="AJ21" s="40" t="n">
-        <v>6464</v>
+        <v>6554.92</v>
       </c>
     </row>
     <row r="22" ht="15.6" customHeight="1" s="37">
@@ -2501,7 +2501,7 @@
         <v>2676</v>
       </c>
       <c r="C22" s="11" t="n">
-        <v>2376</v>
+        <v>2403.77</v>
       </c>
       <c r="D22" s="11" t="n">
         <v>2262</v>
@@ -2540,7 +2540,7 @@
         <v>832</v>
       </c>
       <c r="P22" s="11" t="n">
-        <v>1054</v>
+        <v>1028.34</v>
       </c>
       <c r="Q22" s="11" t="n">
         <v>1047</v>
@@ -2552,7 +2552,7 @@
         <v>1047</v>
       </c>
       <c r="T22" s="11" t="n">
-        <v>193</v>
+        <v>204.58</v>
       </c>
       <c r="U22" s="20" t="n"/>
       <c r="V22" s="20" t="n"/>
@@ -2568,13 +2568,13 @@
       <c r="AF22" s="21" t="n"/>
       <c r="AG22" s="39" t="n"/>
       <c r="AH22" s="40" t="n">
-        <v>3216</v>
+        <v>3142.9</v>
       </c>
       <c r="AI22" s="40" t="n">
-        <v>5632</v>
+        <v>5758.73</v>
       </c>
       <c r="AJ22" s="40" t="n">
-        <v>6265</v>
+        <v>6387.04</v>
       </c>
     </row>
     <row r="23" ht="15.6" customHeight="1" s="37">
@@ -2587,7 +2587,7 @@
         <v>4958</v>
       </c>
       <c r="C23" s="11" t="n">
-        <v>4658</v>
+        <v>4685.6</v>
       </c>
       <c r="D23" s="11" t="n">
         <v>4544</v>
@@ -2626,7 +2626,7 @@
         <v>3114</v>
       </c>
       <c r="P23" s="11" t="n">
-        <v>3336</v>
+        <v>3292.52</v>
       </c>
       <c r="Q23" s="11" t="n">
         <v>3329</v>
@@ -2638,10 +2638,10 @@
         <v>3329</v>
       </c>
       <c r="T23" s="11" t="n">
-        <v>2484</v>
+        <v>2461.71</v>
       </c>
       <c r="U23" s="11" t="n">
-        <v>2303</v>
+        <v>2293.84</v>
       </c>
       <c r="V23" s="20" t="n"/>
       <c r="W23" s="20" t="n"/>
@@ -2656,13 +2656,13 @@
       <c r="AF23" s="21" t="n"/>
       <c r="AG23" s="39" t="n"/>
       <c r="AH23" s="40" t="n">
-        <v>1207</v>
+        <v>1049.09</v>
       </c>
       <c r="AI23" s="40" t="n">
-        <v>3568</v>
+        <v>4019.91</v>
       </c>
       <c r="AJ23" s="40" t="n">
-        <v>4223</v>
+        <v>4637.08</v>
       </c>
     </row>
     <row r="24" ht="15.6" customHeight="1" s="37">
@@ -2675,7 +2675,7 @@
         <v>5307</v>
       </c>
       <c r="C24" s="11" t="n">
-        <v>5007</v>
+        <v>5034.03</v>
       </c>
       <c r="D24" s="11" t="n">
         <v>4892</v>
@@ -2714,7 +2714,7 @@
         <v>3462</v>
       </c>
       <c r="P24" s="11" t="n">
-        <v>3684</v>
+        <v>3632.62</v>
       </c>
       <c r="Q24" s="11" t="n">
         <v>3677</v>
@@ -2726,10 +2726,10 @@
         <v>3677</v>
       </c>
       <c r="T24" s="11" t="n">
-        <v>2833</v>
+        <v>2801.81</v>
       </c>
       <c r="U24" s="11" t="n">
-        <v>2652</v>
+        <v>2633.94</v>
       </c>
       <c r="V24" s="11" t="n">
         <v>454</v>
@@ -2746,13 +2746,13 @@
       <c r="AF24" s="21" t="n"/>
       <c r="AG24" s="39" t="n"/>
       <c r="AH24" s="40" t="n">
-        <v>1143</v>
+        <v>807.8</v>
       </c>
       <c r="AI24" s="40" t="n">
-        <v>3508</v>
+        <v>3914.36</v>
       </c>
       <c r="AJ24" s="40" t="n">
-        <v>4152</v>
+        <v>4502.23</v>
       </c>
     </row>
     <row r="25" ht="15.6" customHeight="1" s="37">
@@ -2762,28 +2762,28 @@
         </is>
       </c>
       <c r="B25" s="11" t="n">
-        <v>6013</v>
+        <v>5994.86</v>
       </c>
       <c r="C25" s="11" t="n">
-        <v>5713</v>
+        <v>5724.76</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>5599</v>
+        <v>5571.59</v>
       </c>
       <c r="E25" s="11" t="n">
         <v>5146</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>4992</v>
+        <v>4946.75</v>
       </c>
       <c r="G25" s="11" t="n">
-        <v>4996</v>
+        <v>4956.12</v>
       </c>
       <c r="H25" s="11" t="n">
         <v>5010</v>
       </c>
       <c r="I25" s="11" t="n">
-        <v>5008</v>
+        <v>4966.68</v>
       </c>
       <c r="J25" s="11" t="n">
         <v>4975</v>
@@ -2804,7 +2804,7 @@
         <v>4169</v>
       </c>
       <c r="P25" s="11" t="n">
-        <v>4391</v>
+        <v>4326.66</v>
       </c>
       <c r="Q25" s="11" t="n">
         <v>4384</v>
@@ -2816,16 +2816,16 @@
         <v>4384</v>
       </c>
       <c r="T25" s="11" t="n">
-        <v>3540</v>
+        <v>3495.85</v>
       </c>
       <c r="U25" s="11" t="n">
-        <v>3359</v>
+        <v>3327.98</v>
       </c>
       <c r="V25" s="11" t="n">
-        <v>1220</v>
+        <v>1284.09</v>
       </c>
       <c r="W25" s="11" t="n">
-        <v>938</v>
+        <v>918.78</v>
       </c>
       <c r="X25" s="20" t="n"/>
       <c r="Y25" s="20" t="n"/>
@@ -2838,13 +2838,13 @@
       <c r="AF25" s="21" t="n"/>
       <c r="AG25" s="39" t="n"/>
       <c r="AH25" s="40" t="n">
-        <v>230</v>
+        <v>232.8</v>
       </c>
       <c r="AI25" s="40" t="n">
-        <v>2344</v>
+        <v>3960.28</v>
       </c>
       <c r="AJ25" s="40" t="n">
-        <v>3001</v>
+        <v>4540.34</v>
       </c>
     </row>
     <row r="26" ht="15.6" customHeight="1" s="37">
@@ -2932,7 +2932,7 @@
       <c r="AF26" s="21" t="n"/>
       <c r="AG26" s="39" t="n"/>
       <c r="AH26" s="40" t="n">
-        <v>1723</v>
+        <v>2190</v>
       </c>
       <c r="AI26" s="40" t="n">
         <v>2222</v>
@@ -3028,7 +3028,7 @@
       <c r="AF27" s="21" t="n"/>
       <c r="AG27" s="39" t="n"/>
       <c r="AH27" s="40" t="n">
-        <v>1887</v>
+        <v>1561</v>
       </c>
       <c r="AI27" s="40" t="n">
         <v>2286</v>
@@ -3126,7 +3126,7 @@
       <c r="AF28" s="21" t="n"/>
       <c r="AG28" s="39" t="n"/>
       <c r="AH28" s="40" t="n">
-        <v>2487</v>
+        <v>2135.7</v>
       </c>
       <c r="AI28" s="40" t="n">
         <v>2041</v>
@@ -3226,7 +3226,7 @@
       <c r="AF29" s="21" t="n"/>
       <c r="AG29" s="39" t="n"/>
       <c r="AH29" s="40" t="n">
-        <v>2439</v>
+        <v>2101.7</v>
       </c>
       <c r="AI29" s="40" t="n">
         <v>1626</v>
@@ -3245,7 +3245,7 @@
         <v>7469</v>
       </c>
       <c r="C30" s="11" t="n">
-        <v>7169</v>
+        <v>7196.56</v>
       </c>
       <c r="D30" s="11" t="n">
         <v>7055</v>
@@ -3284,7 +3284,7 @@
         <v>5624</v>
       </c>
       <c r="P30" s="11" t="n">
-        <v>5847</v>
+        <v>5764.44</v>
       </c>
       <c r="Q30" s="11" t="n">
         <v>5840</v>
@@ -3296,19 +3296,19 @@
         <v>5840</v>
       </c>
       <c r="T30" s="11" t="n">
-        <v>4995</v>
+        <v>4933.63</v>
       </c>
       <c r="U30" s="11" t="n">
-        <v>4814</v>
+        <v>4765.75</v>
       </c>
       <c r="V30" s="11" t="n">
-        <v>2985</v>
+        <v>3015.79</v>
       </c>
       <c r="W30" s="11" t="n">
-        <v>2879</v>
+        <v>2880.94</v>
       </c>
       <c r="X30" s="11" t="n">
-        <v>2919</v>
+        <v>2925.23</v>
       </c>
       <c r="Y30" s="11" t="n">
         <v>1314</v>
@@ -3328,13 +3328,13 @@
       <c r="AF30" s="21" t="n"/>
       <c r="AG30" s="39" t="n"/>
       <c r="AH30" s="40" t="n">
-        <v>3077</v>
+        <v>2733.9</v>
       </c>
       <c r="AI30" s="40" t="n">
-        <v>1044</v>
+        <v>1060.41</v>
       </c>
       <c r="AJ30" s="40" t="n">
-        <v>1757</v>
+        <v>1635.26</v>
       </c>
     </row>
     <row r="31" ht="15.6" customHeight="1" s="37">
@@ -3432,7 +3432,7 @@
       <c r="AF31" s="21" t="n"/>
       <c r="AG31" s="39" t="n"/>
       <c r="AH31" s="40" t="n">
-        <v>3091</v>
+        <v>2747</v>
       </c>
       <c r="AI31" s="40" t="n">
         <v>1041</v>
@@ -3538,7 +3538,7 @@
       <c r="AF32" s="21" t="n"/>
       <c r="AG32" s="39" t="n"/>
       <c r="AH32" s="40" t="n">
-        <v>3342</v>
+        <v>2992.1</v>
       </c>
       <c r="AI32" s="40" t="n">
         <v>1015</v>
@@ -3646,7 +3646,7 @@
       <c r="AF33" s="39" t="n"/>
       <c r="AG33" s="39" t="n"/>
       <c r="AH33" s="40" t="n">
-        <v>3928</v>
+        <v>3622.6</v>
       </c>
       <c r="AI33" s="40" t="n">
         <v>971</v>
@@ -3756,7 +3756,7 @@
       </c>
       <c r="AG34" s="39" t="n"/>
       <c r="AH34" s="40" t="n">
-        <v>4034</v>
+        <v>3755</v>
       </c>
       <c r="AI34" s="40" t="n">
         <v>995</v>
@@ -3772,109 +3772,109 @@
         </is>
       </c>
       <c r="B35" s="40" t="n">
-        <v>3641</v>
+        <v>5809.8</v>
       </c>
       <c r="C35" s="40" t="n">
-        <v>3754</v>
+        <v>5539.6</v>
       </c>
       <c r="D35" s="40" t="n">
-        <v>3777</v>
+        <v>5386.5</v>
       </c>
       <c r="E35" s="40" t="n">
-        <v>3664</v>
+        <v>4879.1</v>
       </c>
       <c r="F35" s="40" t="n">
-        <v>3477</v>
+        <v>4761.6</v>
       </c>
       <c r="G35" s="40" t="n">
-        <v>3430</v>
+        <v>4771</v>
       </c>
       <c r="H35" s="40" t="n">
-        <v>3431</v>
+        <v>4907.3</v>
       </c>
       <c r="I35" s="40" t="n">
-        <v>3424</v>
+        <v>4781.6</v>
       </c>
       <c r="J35" s="40" t="n">
-        <v>3472</v>
+        <v>4766.3</v>
       </c>
       <c r="K35" s="40" t="n">
-        <v>3856</v>
+        <v>5128.4</v>
       </c>
       <c r="L35" s="40" t="n">
-        <v>3864</v>
+        <v>5128.4</v>
       </c>
       <c r="M35" s="40" t="n">
-        <v>3811</v>
+        <v>5036</v>
       </c>
       <c r="N35" s="40" t="n">
-        <v>3828</v>
+        <v>4936.2</v>
       </c>
       <c r="O35" s="40" t="n">
-        <v>3284</v>
+        <v>3976</v>
       </c>
       <c r="P35" s="40" t="n">
-        <v>2879</v>
+        <v>4141.6</v>
       </c>
       <c r="Q35" s="40" t="n">
-        <v>2840</v>
+        <v>4214.8</v>
       </c>
       <c r="R35" s="40" t="n">
-        <v>2847</v>
+        <v>4198</v>
       </c>
       <c r="S35" s="40" t="n">
-        <v>2848</v>
+        <v>3838</v>
       </c>
       <c r="T35" s="40" t="n">
-        <v>3415</v>
+        <v>3310.7</v>
       </c>
       <c r="U35" s="40" t="n">
-        <v>3216</v>
+        <v>3142.9</v>
       </c>
       <c r="V35" s="40" t="n">
-        <v>1207</v>
+        <v>1049.09</v>
       </c>
       <c r="W35" s="40" t="n">
-        <v>1143</v>
+        <v>807.8</v>
       </c>
       <c r="X35" s="40" t="n">
-        <v>230</v>
+        <v>232.8</v>
       </c>
       <c r="Y35" s="40" t="n">
-        <v>1723</v>
+        <v>2190</v>
       </c>
       <c r="Z35" s="40" t="n">
-        <v>1887</v>
+        <v>1561</v>
       </c>
       <c r="AA35" s="40" t="n">
-        <v>2487</v>
+        <v>2135.7</v>
       </c>
       <c r="AB35" s="40" t="n">
-        <v>2439</v>
+        <v>2101.7</v>
       </c>
       <c r="AC35" s="40" t="n">
-        <v>3077</v>
+        <v>2733.9</v>
       </c>
       <c r="AD35" s="40" t="n">
-        <v>3091</v>
+        <v>2747</v>
       </c>
       <c r="AE35" s="40" t="n">
-        <v>3342</v>
+        <v>2992.1</v>
       </c>
       <c r="AF35" s="40" t="n">
-        <v>3928</v>
+        <v>3622.6</v>
       </c>
       <c r="AG35" s="40" t="n">
-        <v>4034</v>
+        <v>3755</v>
       </c>
       <c r="AH35" s="40" t="n">
         <v>0</v>
       </c>
       <c r="AI35" s="40" t="n">
-        <v>2416</v>
+        <v>3768.8</v>
       </c>
       <c r="AJ35" s="40" t="n">
-        <v>3068</v>
+        <v>4348.8</v>
       </c>
     </row>
     <row r="36" ht="15.6" customHeight="1" s="37">
@@ -3884,28 +3884,28 @@
         </is>
       </c>
       <c r="B36" s="40" t="n">
-        <v>5430</v>
+        <v>8503.450000000001</v>
       </c>
       <c r="C36" s="40" t="n">
-        <v>5664</v>
+        <v>8230.93</v>
       </c>
       <c r="D36" s="40" t="n">
-        <v>5720</v>
+        <v>8089.3</v>
       </c>
       <c r="E36" s="40" t="n">
         <v>5758</v>
       </c>
       <c r="F36" s="40" t="n">
-        <v>5641</v>
+        <v>7481.7</v>
       </c>
       <c r="G36" s="40" t="n">
-        <v>5595</v>
+        <v>7485.87</v>
       </c>
       <c r="H36" s="40" t="n">
         <v>5594</v>
       </c>
       <c r="I36" s="40" t="n">
-        <v>5582</v>
+        <v>7497.93</v>
       </c>
       <c r="J36" s="40" t="n">
         <v>5641</v>
@@ -3926,7 +3926,7 @@
         <v>5652</v>
       </c>
       <c r="P36" s="40" t="n">
-        <v>5253</v>
+        <v>6757.42</v>
       </c>
       <c r="Q36" s="40" t="n">
         <v>5210</v>
@@ -3938,19 +3938,19 @@
         <v>5220</v>
       </c>
       <c r="T36" s="40" t="n">
-        <v>5830</v>
+        <v>5926.6</v>
       </c>
       <c r="U36" s="40" t="n">
-        <v>5632</v>
+        <v>5758.73</v>
       </c>
       <c r="V36" s="40" t="n">
-        <v>3568</v>
+        <v>4019.91</v>
       </c>
       <c r="W36" s="40" t="n">
-        <v>3508</v>
+        <v>3914.36</v>
       </c>
       <c r="X36" s="40" t="n">
-        <v>2344</v>
+        <v>3960.28</v>
       </c>
       <c r="Y36" s="40" t="n">
         <v>2222</v>
@@ -3965,7 +3965,7 @@
         <v>1626</v>
       </c>
       <c r="AC36" s="40" t="n">
-        <v>1044</v>
+        <v>1060.41</v>
       </c>
       <c r="AD36" s="40" t="n">
         <v>1041</v>
@@ -3980,13 +3980,13 @@
         <v>995</v>
       </c>
       <c r="AH36" s="40" t="n">
-        <v>2416</v>
+        <v>3768.8</v>
       </c>
       <c r="AI36" s="40" t="n">
         <v>0</v>
       </c>
       <c r="AJ36" s="40" t="n">
-        <v>748</v>
+        <v>766.51</v>
       </c>
     </row>
     <row r="37" ht="15.6" customHeight="1" s="37">
@@ -3996,28 +3996,28 @@
         </is>
       </c>
       <c r="B37" s="40" t="n">
-        <v>5736</v>
+        <v>9083.51</v>
       </c>
       <c r="C37" s="40" t="n">
-        <v>6004</v>
+        <v>8810.98</v>
       </c>
       <c r="D37" s="40" t="n">
-        <v>6071</v>
+        <v>8669.360000000001</v>
       </c>
       <c r="E37" s="40" t="n">
         <v>6173</v>
       </c>
       <c r="F37" s="40" t="n">
-        <v>6093</v>
+        <v>8061.75</v>
       </c>
       <c r="G37" s="40" t="n">
-        <v>6049</v>
+        <v>8065.93</v>
       </c>
       <c r="H37" s="40" t="n">
         <v>6048</v>
       </c>
       <c r="I37" s="40" t="n">
-        <v>6034</v>
+        <v>8077.99</v>
       </c>
       <c r="J37" s="40" t="n">
         <v>6095</v>
@@ -4038,7 +4038,7 @@
         <v>6223</v>
       </c>
       <c r="P37" s="40" t="n">
-        <v>5834</v>
+        <v>7385.73</v>
       </c>
       <c r="Q37" s="40" t="n">
         <v>5789</v>
@@ -4050,19 +4050,19 @@
         <v>5799</v>
       </c>
       <c r="T37" s="40" t="n">
-        <v>6464</v>
+        <v>6554.92</v>
       </c>
       <c r="U37" s="40" t="n">
-        <v>6265</v>
+        <v>6387.04</v>
       </c>
       <c r="V37" s="40" t="n">
-        <v>4223</v>
+        <v>4637.08</v>
       </c>
       <c r="W37" s="40" t="n">
-        <v>4152</v>
+        <v>4502.23</v>
       </c>
       <c r="X37" s="40" t="n">
-        <v>3001</v>
+        <v>4540.34</v>
       </c>
       <c r="Y37" s="40" t="n">
         <v>2938</v>
@@ -4077,7 +4077,7 @@
         <v>2271</v>
       </c>
       <c r="AC37" s="40" t="n">
-        <v>1757</v>
+        <v>1635.26</v>
       </c>
       <c r="AD37" s="40" t="n">
         <v>1755</v>
@@ -4092,10 +4092,10 @@
         <v>1457</v>
       </c>
       <c r="AH37" s="40" t="n">
-        <v>3068</v>
+        <v>4348.8</v>
       </c>
       <c r="AI37" s="40" t="n">
-        <v>748</v>
+        <v>766.51</v>
       </c>
       <c r="AJ37" s="40" t="n">
         <v>0</v>
@@ -8042,8 +8042,6 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="67"/>
-    <row r="68"/>
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
@@ -11694,7 +11692,7 @@
       <c r="E265" s="5" t="n">
         <v>12.5</v>
       </c>
-      <c r="F265" t="n">
+      <c r="F265" s="0" t="n">
         <v>1.2</v>
       </c>
     </row>
@@ -11715,7 +11713,7 @@
       <c r="E266" s="5" t="n">
         <v>15.5</v>
       </c>
-      <c r="F266" t="n">
+      <c r="F266" s="0" t="n">
         <v>1.2</v>
       </c>
     </row>
@@ -11736,7 +11734,7 @@
       <c r="E267" s="5" t="n">
         <v>18</v>
       </c>
-      <c r="F267" t="n">
+      <c r="F267" s="0" t="n">
         <v>1.2</v>
       </c>
     </row>

</xml_diff>